<commit_message>
fix: resolve student name column detection when № sequence column exists
</commit_message>
<xml_diff>
--- a/EduFinance_Moliya_Shabloni.xlsx
+++ b/EduFinance_Moliya_Shabloni.xlsx
@@ -1,16 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <workbookPr/>
+  <bookViews>
+    <workbookView windowWidth="23040" windowHeight="9708" activeTab="3"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="To'lovlar" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="O'qituvchilar Oyligi" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Markaz Xarajatlari" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="Founder Xarajatlari" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="Moliya Xulosasi" state="visible" r:id="rId8"/>
+    <sheet name="To'lovlar" sheetId="1" r:id="rId1"/>
+    <sheet name="O'qituvchilar Oyligi" sheetId="2" r:id="rId2"/>
+    <sheet name="Markaz Xarajatlari" sheetId="3" r:id="rId3"/>
+    <sheet name="Founder Xarajatlari" sheetId="4" r:id="rId4"/>
+    <sheet name="Moliya Xulosasi" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -377,39 +393,206 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="#,##0 &quot;so'm&quot;"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="5">
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="178" formatCode="#,##0\ &quot;so'm&quot;"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="25">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
-      <family val="2"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
+      <color rgb="FF047857"/>
       <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF047857"/>
+      <sz val="11"/>
+      <color rgb="FFB91C1C"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFB91C1C"/>
+      <sz val="12"/>
+      <color rgb="FF15803D"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF15803D"/>
-      <sz val="12"/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="38">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -418,31 +601,222 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF334155"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF6D28D9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD97706"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1D4ED8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FF047857"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF1D4ED8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD97706"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF6D28D9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF334155"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -465,91 +839,377 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="176" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="178" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="178" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="178" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="178" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="178" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="178" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -871,895 +1531,908 @@
       </a:style>
     </a:lnDef>
   </a:objectDefaults>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr>
     <tabColor rgb="FF10B981"/>
   </sheetPr>
   <dimension ref="A1:K6"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="5"/>
   <cols>
-    <col min="1" max="1" width="6" style="1" customWidth="1"/>
+    <col min="1" max="1" width="6" style="15" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="4" width="18" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="16" style="2" customWidth="1"/>
-    <col min="7" max="8" width="15" style="2" customWidth="1"/>
-    <col min="9" max="9" width="16" style="2" customWidth="1"/>
-    <col min="10" max="10" width="15" style="1" customWidth="1"/>
+    <col min="6" max="6" width="16" style="4" customWidth="1"/>
+    <col min="7" max="8" width="15" style="4" customWidth="1"/>
+    <col min="9" max="9" width="16" style="4" customWidth="1"/>
+    <col min="10" max="10" width="15" style="15" customWidth="1"/>
     <col min="11" max="11" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" ht="28" customHeight="1" spans="1:11">
+      <c r="A1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="26" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="5">
+    <row r="2" spans="1:11">
+      <c r="A2" s="18">
         <v>1</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="F2" s="7">
+      <c r="F2" s="10">
         <v>750000</v>
       </c>
-      <c r="G2" s="7">
+      <c r="G2" s="10">
         <v>400000</v>
       </c>
-      <c r="H2" s="7">
+      <c r="H2" s="10">
         <v>350000</v>
       </c>
-      <c r="I2" s="7">
+      <c r="I2" s="10">
         <f>F2-(G2+H2)</f>
-      </c>
-      <c r="J2" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="J2" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="K2" s="6" t="s">
+      <c r="K2" s="9" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="5">
+    <row r="3" spans="1:11">
+      <c r="A3" s="18">
         <v>2</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="7">
+      <c r="F3" s="10">
         <v>800000</v>
       </c>
-      <c r="G3" s="7">
+      <c r="G3" s="10">
         <v>0</v>
       </c>
-      <c r="H3" s="7">
+      <c r="H3" s="10">
         <v>0</v>
       </c>
-      <c r="I3" s="7">
+      <c r="I3" s="10">
         <f>F3-(G3+H3)</f>
-      </c>
-      <c r="J3" s="5" t="s">
+        <v>800000</v>
+      </c>
+      <c r="J3" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="K3" s="6" t="s">
+      <c r="K3" s="9" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="5">
+    <row r="4" spans="1:11">
+      <c r="A4" s="18">
         <v>3</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="F4" s="7">
+      <c r="F4" s="10">
         <v>750000</v>
       </c>
-      <c r="G4" s="7">
+      <c r="G4" s="10">
         <v>500000</v>
       </c>
-      <c r="H4" s="7">
+      <c r="H4" s="10">
         <v>0</v>
       </c>
-      <c r="I4" s="7">
+      <c r="I4" s="10">
         <f>F4-(G4+H4)</f>
-      </c>
-      <c r="J4" s="5" t="s">
+        <v>250000</v>
+      </c>
+      <c r="J4" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="K4" s="6" t="s">
+      <c r="K4" s="9" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="5">
+    <row r="5" spans="1:11">
+      <c r="A5" s="18">
         <v>4</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5" s="10">
         <v>700000</v>
       </c>
-      <c r="G5" s="7">
+      <c r="G5" s="10">
         <v>0</v>
       </c>
-      <c r="H5" s="7">
+      <c r="H5" s="10">
         <v>700000</v>
       </c>
-      <c r="I5" s="7">
+      <c r="I5" s="10">
         <f>F5-(G5+H5)</f>
-      </c>
-      <c r="J5" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="J5" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="K5" s="6" t="s">
+      <c r="K5" s="9" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="5">
+    <row r="6" spans="1:11">
+      <c r="A6" s="18">
         <v>5</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="F6" s="7">
+      <c r="F6" s="10">
         <v>650000</v>
       </c>
-      <c r="G6" s="7">
+      <c r="G6" s="10">
         <v>1950000</v>
       </c>
-      <c r="H6" s="7">
+      <c r="H6" s="10">
         <v>0</v>
       </c>
-      <c r="I6" s="7">
+      <c r="I6" s="10">
         <f>F6-(G6+H6)</f>
-      </c>
-      <c r="J6" s="5" t="s">
+        <v>-1300000</v>
+      </c>
+      <c r="J6" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="K6" s="6" t="s">
+      <c r="K6" s="9" t="s">
         <v>40</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup paperSize="1" orientation="portrait"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr>
     <tabColor rgb="FF3B82F6"/>
   </sheetPr>
   <dimension ref="A1:K5"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="1" width="6" style="1" customWidth="1"/>
+    <col min="1" max="1" width="6" style="15" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="20" style="2" customWidth="1"/>
-    <col min="5" max="5" width="15" style="8" customWidth="1"/>
-    <col min="6" max="6" width="16" style="2" customWidth="1"/>
-    <col min="7" max="7" width="18" style="2" customWidth="1"/>
-    <col min="8" max="8" width="16" style="2" customWidth="1"/>
-    <col min="9" max="9" width="22" style="2" customWidth="1"/>
-    <col min="10" max="10" width="15" style="1" customWidth="1"/>
+    <col min="4" max="4" width="20" style="4" customWidth="1"/>
+    <col min="5" max="5" width="15" style="21" customWidth="1"/>
+    <col min="6" max="6" width="16" style="4" customWidth="1"/>
+    <col min="7" max="7" width="18" style="4" customWidth="1"/>
+    <col min="8" max="8" width="16" style="4" customWidth="1"/>
+    <col min="9" max="9" width="22" style="4" customWidth="1"/>
+    <col min="10" max="10" width="15" style="15" customWidth="1"/>
     <col min="11" max="11" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+    <row r="1" ht="28" customHeight="1" spans="1:11">
+      <c r="A1" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="F1" s="23" t="s">
         <v>45</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="G1" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="H1" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="I1" s="10" t="s">
+      <c r="I1" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="J1" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="K1" s="22" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="5">
+    <row r="2" spans="1:11">
+      <c r="A2" s="18">
         <v>1</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="D2" s="7">
+      <c r="D2" s="10">
         <v>6000000</v>
       </c>
-      <c r="E2" s="12">
+      <c r="E2" s="25">
         <v>0.4</v>
       </c>
-      <c r="F2" s="7">
+      <c r="F2" s="10">
         <v>1500000</v>
       </c>
-      <c r="G2" s="7">
+      <c r="G2" s="10">
         <v>0</v>
       </c>
-      <c r="H2" s="7">
+      <c r="H2" s="10">
         <v>200000</v>
       </c>
-      <c r="I2" s="7">
+      <c r="I2" s="10">
         <f>D2+G2-F2-H2</f>
-      </c>
-      <c r="J2" s="5" t="s">
+        <v>4300000</v>
+      </c>
+      <c r="J2" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="K2" s="6" t="s">
+      <c r="K2" s="9" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="5">
+    <row r="3" spans="1:11">
+      <c r="A3" s="18">
         <v>2</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="D3" s="7">
+      <c r="D3" s="10">
         <v>3500000</v>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="25">
         <v>0</v>
       </c>
-      <c r="F3" s="7">
+      <c r="F3" s="10">
         <v>500000</v>
       </c>
-      <c r="G3" s="7">
+      <c r="G3" s="10">
         <v>0</v>
       </c>
-      <c r="H3" s="7">
+      <c r="H3" s="10">
         <v>150000</v>
       </c>
-      <c r="I3" s="7">
+      <c r="I3" s="10">
         <f>D3+G3-F3-H3</f>
-      </c>
-      <c r="J3" s="5" t="s">
+        <v>2850000</v>
+      </c>
+      <c r="J3" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="K3" s="6" t="s">
+      <c r="K3" s="9" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="5">
+    <row r="4" spans="1:11">
+      <c r="A4" s="18">
         <v>3</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="D4" s="7">
+      <c r="D4" s="10">
         <v>5500000</v>
       </c>
-      <c r="E4" s="12">
+      <c r="E4" s="25">
         <v>0.4</v>
       </c>
-      <c r="F4" s="7">
+      <c r="F4" s="10">
         <v>1000000</v>
       </c>
-      <c r="G4" s="7">
+      <c r="G4" s="10">
         <v>0</v>
       </c>
-      <c r="H4" s="7">
+      <c r="H4" s="10">
         <v>200000</v>
       </c>
-      <c r="I4" s="7">
+      <c r="I4" s="10">
         <f>D4+G4-F4-H4</f>
-      </c>
-      <c r="J4" s="5" t="s">
+        <v>4300000</v>
+      </c>
+      <c r="J4" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="K4" s="6" t="s">
+      <c r="K4" s="9" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="5">
+    <row r="5" spans="1:11">
+      <c r="A5" s="18">
         <v>4</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="10">
         <v>2000000</v>
       </c>
-      <c r="E5" s="12">
+      <c r="E5" s="25">
         <v>0</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5" s="10">
         <v>0</v>
       </c>
-      <c r="G5" s="7">
+      <c r="G5" s="10">
         <v>0</v>
       </c>
-      <c r="H5" s="7">
+      <c r="H5" s="10">
         <v>50000</v>
       </c>
-      <c r="I5" s="7">
+      <c r="I5" s="10">
         <f>D5+G5-F5-H5</f>
-      </c>
-      <c r="J5" s="5" t="s">
+        <v>1950000</v>
+      </c>
+      <c r="J5" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="K5" s="6" t="s">
+      <c r="K5" s="9" t="s">
         <v>52</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup paperSize="1" orientation="portrait"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr>
     <tabColor rgb="FFF59E0B"/>
   </sheetPr>
   <dimension ref="A1:G7"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="6" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="6" style="1" customWidth="1"/>
-    <col min="2" max="2" width="14" style="1" customWidth="1"/>
+    <col min="1" max="1" width="6" style="15" customWidth="1"/>
+    <col min="2" max="2" width="14" style="15" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="25" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="18" style="2" customWidth="1"/>
-    <col min="7" max="7" width="16" style="1" customWidth="1"/>
+    <col min="6" max="6" width="18" style="4" customWidth="1"/>
+    <col min="7" max="7" width="16" style="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+    <row r="1" ht="28" customHeight="1" spans="1:7">
+      <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="F1" s="14" t="s">
+      <c r="F1" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="G1" s="19" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="5">
+    <row r="2" spans="1:7">
+      <c r="A2" s="18">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="F2" s="7">
+      <c r="F2" s="10">
         <v>12000000</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="G2" s="18" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="5">
+    <row r="3" spans="1:7">
+      <c r="A3" s="18">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="F3" s="7">
+      <c r="F3" s="10">
         <v>1850000</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="18" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="5">
+    <row r="4" spans="1:7">
+      <c r="A4" s="18">
         <v>3</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="F4" s="7">
+      <c r="F4" s="10">
         <v>450000</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="18" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="5">
+    <row r="5" spans="1:7">
+      <c r="A5" s="18">
         <v>4</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5" s="10">
         <v>2500000</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="18" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="5">
+    <row r="6" spans="1:7">
+      <c r="A6" s="18">
         <v>5</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="F6" s="7">
+      <c r="F6" s="10">
         <v>350000</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="G6" s="18" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="5">
+    <row r="7" spans="1:7">
+      <c r="A7" s="18">
         <v>6</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="F7" s="7">
+      <c r="F7" s="10">
         <v>180000</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="G7" s="18" t="s">
         <v>6</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup paperSize="1" orientation="portrait"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr>
     <tabColor rgb="FF8B5CF6"/>
   </sheetPr>
   <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="5" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="6" style="1" customWidth="1"/>
-    <col min="2" max="2" width="14" style="1" customWidth="1"/>
+    <col min="1" max="1" width="6" style="15" customWidth="1"/>
+    <col min="2" max="2" width="14" style="15" customWidth="1"/>
     <col min="3" max="3" width="25" customWidth="1"/>
     <col min="4" max="4" width="24" customWidth="1"/>
     <col min="5" max="5" width="32" customWidth="1"/>
-    <col min="6" max="6" width="18" style="2" customWidth="1"/>
-    <col min="7" max="7" width="16" style="1" customWidth="1"/>
+    <col min="6" max="6" width="18" style="4" customWidth="1"/>
+    <col min="7" max="7" width="16" style="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+    <row r="1" ht="28" customHeight="1" spans="1:7">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="16" t="s">
         <v>86</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="E1" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="F1" s="16" t="s">
+      <c r="F1" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="G1" s="15" t="s">
+      <c r="G1" s="16" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="5">
+    <row r="2" spans="1:7">
+      <c r="A2" s="18">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="F2" s="7">
+      <c r="F2" s="10">
         <v>500000</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="G2" s="18" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="5">
+    <row r="3" spans="1:7">
+      <c r="A3" s="18">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="F3" s="7">
+      <c r="F3" s="10">
         <v>500000</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="18" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="5">
+    <row r="4" spans="1:7">
+      <c r="A4" s="18">
         <v>3</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="F4" s="7">
+      <c r="F4" s="10">
         <v>500000</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="18" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="5">
+    <row r="5" spans="1:7">
+      <c r="A5" s="18">
         <v>4</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5" s="10">
         <v>200000</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="18" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="5">
+    <row r="6" spans="1:7">
+      <c r="A6" s="18">
         <v>5</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="18" t="s">
         <v>98</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="F6" s="7">
+      <c r="F6" s="10">
         <v>2000000</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="G6" s="18" t="s">
         <v>73</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup paperSize="1" orientation="portrait"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr>
     <tabColor rgb="FF475569"/>
   </sheetPr>
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="7" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="35" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
-    <col min="3" max="3" width="22" style="2" customWidth="1"/>
+    <col min="3" max="3" width="22" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+    <row r="1" ht="28" customHeight="1" spans="1:3">
+      <c r="A1" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="C1" s="6" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="2" spans="1:3" s="19" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
+    <row r="2" s="1" customFormat="1" spans="1:3">
+      <c r="A2" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="C2" s="21">
-        <f>SUM('To'lovlar'!G2:H1000)</f>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+      <c r="C2" s="8"/>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="C3" s="7">
-        <f>SUM('O'qituvchilar Oyligi'!I2:I1000)</f>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="C3" s="10"/>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4" s="10">
         <f>SUM('Markaz Xarajatlari'!F2:F1000)</f>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+        <v>17330000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="C5" s="7">
+      <c r="C5" s="10">
         <f>SUM('Founder Xarajatlari'!F2:F1000)</f>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
+        <v>3700000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="10" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="7" spans="1:3" s="22" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="23" t="s">
+    <row r="7" s="2" customFormat="1" spans="1:3">
+      <c r="A7" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="B7" s="23" t="s">
+      <c r="B7" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="C7" s="24">
+      <c r="C7" s="12">
         <f>C3+C4+C5</f>
-      </c>
-    </row>
-    <row r="8" spans="1:3" s="25" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="26" t="s">
+        <v>21030000</v>
+      </c>
+    </row>
+    <row r="8" s="3" customFormat="1" ht="15.6" spans="1:3">
+      <c r="A8" s="13" t="s">
         <v>117</v>
       </c>
-      <c r="B8" s="26" t="s">
+      <c r="B8" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="C8" s="27">
+      <c r="C8" s="14">
         <f>C2-C7</f>
+        <v>-21030000</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup paperSize="1" orientation="portrait"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>